<commit_message>
Daily knowledge base backup | 2026-03-10 00:00 +05 | 2026-03-09 19:00 UTC
</commit_message>
<xml_diff>
--- a/Таблица_для_задачи_демо_заполнено.xlsx
+++ b/Таблица_для_задачи_демо_заполнено.xlsx
@@ -486,9 +486,9 @@
       <c r="C4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="1" t="n"/>
-      <c r="F4" s="1" t="n"/>
-      <c r="G4" s="1" t="n"/>
+      <c r="D4" s="1" t="inlineStr"/>
+      <c r="F4" s="1" t="inlineStr"/>
+      <c r="G4" s="1" t="inlineStr"/>
       <c r="H4">
         <f>3000*G4</f>
         <v/>
@@ -505,7 +505,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Головка шарнирная Festo SGS-M20x1,5 с шестигранной гайкой для сферического поворотного крепления цилиндров Festo серий DSBC, DSBG, DNC (9264)</t>
+          <t>Головка шарнирная Festo SGS-M20x1,5 (9264)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -516,15 +516,26 @@
       <c r="C5" t="n">
         <v>2</v>
       </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
       <c r="H5">
         <f>3000*G5</f>
         <v/>
       </c>
+      <c r="I5">
+        <f>(E5+H5+(E5+H5)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J5">
+        <f>I5*C5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Распределитель Festo CPE14-M1BH-5L-1/8 с электроуправлением 8 бар 800 л/мин (196941)</t>
+          <t>Распределитель Festo CPE14-M1BH-5L-1/8 (196941)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -535,10 +546,21 @@
       <c r="C6" t="n">
         <v>2</v>
       </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6">
         <f>3000*G6</f>
         <v/>
       </c>
+      <c r="I6">
+        <f>(E6+H6+(E6+H6)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J6">
+        <f>I6*C6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -554,15 +576,26 @@
       <c r="C7" t="n">
         <v>1</v>
       </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
       <c r="H7">
         <f>3000*G7</f>
         <v/>
       </c>
+      <c r="I7">
+        <f>(E7+H7+(E7+H7)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J7">
+        <f>I7*C7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Патрон стопорный Festo KP-25-5000 ф25 (178460)</t>
+          <t>Патрон стопорный Festo KP-25-5000 (178460)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -573,15 +606,26 @@
       <c r="C8" t="n">
         <v>2</v>
       </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8">
         <f>3000*G8</f>
         <v/>
       </c>
+      <c r="I8">
+        <f>(E8+H8+(E8+H8)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>I8*C8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Розетка штекерная с кабелем Festo KME-1-24DC-5-LED 4 А 24 В 3-pin тип C IP67 (30945)</t>
+          <t>Розетка штекерная с кабелем Festo KME-1-24DC-5-LED (30945)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -592,15 +636,26 @@
       <c r="C9" t="n">
         <v>4</v>
       </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
       <c r="H9">
         <f>3000*G9</f>
         <v/>
       </c>
+      <c r="I9">
+        <f>(E9+H9+(E9+H9)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J9">
+        <f>I9*C9</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Распределитель Festo MPYE-5-3/8-010-B с пропорциональным управлением 10 бар 2000 л/мин (151695)</t>
+          <t>Распределитель Festo MPYE-5-3/8-010-B (151695)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -611,15 +666,26 @@
       <c r="C10" t="n">
         <v>1</v>
       </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
       <c r="H10">
         <f>3000*G10</f>
         <v/>
       </c>
+      <c r="I10">
+        <f>(E10+H10+(E10+H10)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J10">
+        <f>I10*C10</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Распределитель Festo MFH-5-1/8-B с электроуправлением 10 бар 750 л/мин (19758)</t>
+          <t>Распределитель Festo MFH-5-1/8-B (19758)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -630,15 +696,26 @@
       <c r="C11" t="n">
         <v>7</v>
       </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
       <c r="H11">
         <f>3000*G11</f>
         <v/>
       </c>
+      <c r="I11">
+        <f>(E11+H11+(E11+H11)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J11">
+        <f>I11*C11</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Плита Festo PRS-1/8-7-BB для блочного монтажа (30547)</t>
+          <t>Плита Festo PRS-1/8-7-BB (30547)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -649,15 +726,26 @@
       <c r="C12" t="n">
         <v>1</v>
       </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
       <c r="H12">
         <f>3000*G12</f>
         <v/>
       </c>
+      <c r="I12">
+        <f>(E12+H12+(E12+H12)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J12">
+        <f>I12*C12</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Катушка электромагнитная со стандартной штекерной розеткой Festo MSFW-110-50/60 110 В AC IP65 (6720)</t>
+          <t>Катушка электромагнитная Festo MSFW-110-50/60 (6720)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -668,15 +756,26 @@
       <c r="C13" t="n">
         <v>10</v>
       </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
       <c r="H13">
         <f>3000*G13</f>
         <v/>
       </c>
+      <c r="I13">
+        <f>(E13+H13+(E13+H13)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J13">
+        <f>I13*C13</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Датчик-реле давления Festo PEV-1/4-B 1-12 бар (10773)</t>
+          <t>Датчик-реле давления Festo PEV-1/4-B (10773)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,15 +786,26 @@
       <c r="C14" t="n">
         <v>4</v>
       </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
       <c r="H14">
         <f>3000*G14</f>
         <v/>
       </c>
+      <c r="I14">
+        <f>(E14+H14+(E14+H14)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J14">
+        <f>I14*C14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Модуль электронный Festo VMPA2-FB-EMG-4 для пневмоострова MPA-S (537984)</t>
+          <t>Модуль электронный Festo VMPA2-FB-EMG-4 (537984)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -706,15 +816,26 @@
       <c r="C15" t="n">
         <v>1</v>
       </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
       <c r="H15">
         <f>3000*G15</f>
         <v/>
       </c>
+      <c r="I15">
+        <f>(E15+H15+(E15+H15)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J15">
+        <f>I15*C15</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Распределитель с электроуправлением FESTO VMPA2-M1H-M-PI (537952)</t>
+          <t>Распределитель FESTO VMPA2-M1H-M-PI (537952)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -725,10 +846,21 @@
       <c r="C16" t="n">
         <v>1</v>
       </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
       <c r="H16">
         <f>3000*G16</f>
         <v/>
       </c>
+      <c r="I16">
+        <f>(E16+H16+(E16+H16)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J16">
+        <f>I16*C16</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -744,10 +876,21 @@
       <c r="C17" t="n">
         <v>4</v>
       </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
       <c r="H17">
         <f>3000*G17</f>
         <v/>
       </c>
+      <c r="I17">
+        <f>(E17+H17+(E17+H17)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J17">
+        <f>I17*C17</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -763,15 +906,26 @@
       <c r="C18" t="n">
         <v>4</v>
       </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18">
         <f>3000*G18</f>
         <v/>
       </c>
+      <c r="I18">
+        <f>(E18+H18+(E18+H18)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J18">
+        <f>I18*C18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Датчик положения аналоговый Festo SDAT-MHS-M50-1L-SA-E-0.3-M8 50 мм 1000 Гц PNP (1531265)</t>
+          <t>Датчик положения аналоговый Festo SDAT-MHS-M50-1L-SA-E-0.3-M8 (1531265)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -782,15 +936,26 @@
       <c r="C19" t="n">
         <v>1</v>
       </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19">
         <f>3000*G19</f>
         <v/>
       </c>
+      <c r="I19">
+        <f>(E19+H19+(E19+H19)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J19">
+        <f>I19*C19</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Розетка сетевого питания прямая Festo NECU-G78G5-C2 8 А 250 В 5-pin (543107)</t>
+          <t>Розетка сетевого питания прямая Festo NECU-G78G5-C2 (543107)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -801,15 +966,26 @@
       <c r="C20" t="n">
         <v>2</v>
       </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20">
         <f>3000*G20</f>
         <v/>
       </c>
+      <c r="I20">
+        <f>(E20+H20+(E20+H20)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J20">
+        <f>I20*C20</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Штекер Festo FBS-RJ45-PP-GS 5х72х22 для пневмоостровов (552000)</t>
+          <t>Штекер Festo FBS-RJ45-PP-GS (552000)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -820,10 +996,21 @@
       <c r="C21" t="n">
         <v>6</v>
       </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21">
         <f>3000*G21</f>
         <v/>
       </c>
+      <c r="I21">
+        <f>(E21+H21+(E21+H21)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J21">
+        <f>I21*C21</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -839,15 +1026,26 @@
       <c r="C22" t="n">
         <v>2</v>
       </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
       <c r="H22">
         <f>3000*G22</f>
         <v/>
       </c>
+      <c r="I22">
+        <f>(E22+H22+(E22+H22)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J22">
+        <f>I22*C22</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Клапан пережимной с пневмоуправлением Festo VZQA-C-M22U-6-GG-V4V4E-4 Ду 6 мм Ру 4 бар G1/4" NO 0,7 м3/ч (2931678)</t>
+          <t>Клапан пережимной Festo VZQA-C-M22U-6-GG-V4V4E-4 (2931678)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -858,8 +1056,19 @@
       <c r="C23" t="n">
         <v>1</v>
       </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23">
         <f>3000*G23</f>
+        <v/>
+      </c>
+      <c r="I23">
+        <f>(E23+H23+(E23+H23)*0.2)*1.22</f>
+        <v/>
+      </c>
+      <c r="J23">
+        <f>I23*C23</f>
         <v/>
       </c>
     </row>

</xml_diff>